<commit_message>
updated municipal zoning workbook
</commit_message>
<xml_diff>
--- a/Municipal_Zoning_Workbook.xlsx
+++ b/Municipal_Zoning_Workbook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/055abc5dbe1424b0/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="162" documentId="8_{3E8B709B-7093-42E6-92D8-1867EF89E086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CAAA2FB-7BDA-4C60-9EEC-47FADADF17BA}"/>
+  <xr:revisionPtr revIDLastSave="169" documentId="8_{3E8B709B-7093-42E6-92D8-1867EF89E086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE3BA393-8A6B-44F3-BDDA-BBC57A4AB012}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="7" xr2:uid="{CA185F06-9CD4-4691-B86E-FBA6669FCB7C}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{CA185F06-9CD4-4691-B86E-FBA6669FCB7C}"/>
   </bookViews>
   <sheets>
     <sheet name="City of Frederick" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="227">
   <si>
     <t>Zone</t>
   </si>
@@ -294,9 +294,6 @@
     <t>The R-5 District is intended to provide for attached single family dwellings on small lots, multi-family dwelling structures, and generally, a variety of residential building types and open spaces to create attractive planned communities.</t>
   </si>
   <si>
-    <t>Mixed-use Village</t>
-  </si>
-  <si>
     <t>MXV-1</t>
   </si>
   <si>
@@ -709,6 +706,24 @@
   </si>
   <si>
     <t>It is the intent of the VI District to provide areas for limited industrial purposes that are not significantly objectionable in terms of noise, odor, fumes, etc., to surrounding properties. The regulations that apply within the district are designed to encourage the formation and continuance of a compatible environment for uses generally classified to be light industrial in nature; protect and reserve undeveloped areas that are suitable for such industries; and discourage encroachment by those residential, commercial, or other uses capable of adversely affecting the basic industrial character of the VI District.</t>
+  </si>
+  <si>
+    <t>Residential (R-1)</t>
+  </si>
+  <si>
+    <t>Residential (R-2)</t>
+  </si>
+  <si>
+    <t>Residential (R-3)</t>
+  </si>
+  <si>
+    <t>Residential (R-5)</t>
+  </si>
+  <si>
+    <t>Mixed-use Village (MXV-1)</t>
+  </si>
+  <si>
+    <t>Mixed-use Village (MXV-2)</t>
   </si>
 </sst>
 </file>
@@ -1374,7 +1389,7 @@
   <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="47.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="255.5703125" customWidth="1"/>
@@ -1424,7 +1439,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>74</v>
+        <v>221</v>
       </c>
       <c r="B4" t="s">
         <v>75</v>
@@ -1438,7 +1453,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>74</v>
+        <v>222</v>
       </c>
       <c r="B5" t="s">
         <v>77</v>
@@ -1452,7 +1467,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>74</v>
+        <v>223</v>
       </c>
       <c r="B6" t="s">
         <v>79</v>
@@ -1466,7 +1481,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>74</v>
+        <v>224</v>
       </c>
       <c r="B7" t="s">
         <v>81</v>
@@ -1480,100 +1495,100 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>225</v>
+      </c>
+      <c r="B8" t="s">
         <v>83</v>
-      </c>
-      <c r="B8" t="s">
-        <v>84</v>
       </c>
       <c r="C8" t="s">
         <v>67</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>83</v>
+        <v>226</v>
       </c>
       <c r="B9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C9" t="s">
         <v>67</v>
       </c>
       <c r="D9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>87</v>
+      </c>
+      <c r="B10" t="s">
         <v>88</v>
-      </c>
-      <c r="B10" t="s">
-        <v>89</v>
       </c>
       <c r="C10" t="s">
         <v>67</v>
       </c>
       <c r="D10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>90</v>
+      </c>
+      <c r="B11" t="s">
         <v>91</v>
-      </c>
-      <c r="B11" t="s">
-        <v>92</v>
       </c>
       <c r="C11" t="s">
         <v>67</v>
       </c>
       <c r="D11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>93</v>
+      </c>
+      <c r="B12" t="s">
         <v>94</v>
-      </c>
-      <c r="B12" t="s">
-        <v>95</v>
       </c>
       <c r="C12" t="s">
         <v>67</v>
       </c>
       <c r="D12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>96</v>
+      </c>
+      <c r="B13" t="s">
         <v>97</v>
-      </c>
-      <c r="B13" t="s">
-        <v>98</v>
       </c>
       <c r="C13" t="s">
         <v>67</v>
       </c>
       <c r="D13" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>99</v>
+      </c>
+      <c r="B14" t="s">
         <v>100</v>
-      </c>
-      <c r="B14" t="s">
-        <v>101</v>
       </c>
       <c r="C14" t="s">
         <v>67</v>
       </c>
       <c r="D14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1615,38 +1630,38 @@
         <v>68</v>
       </c>
       <c r="C2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D2" t="s">
         <v>103</v>
-      </c>
-      <c r="D2" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B3" t="s">
         <v>105</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D3" t="s">
         <v>106</v>
-      </c>
-      <c r="C3" t="s">
-        <v>103</v>
-      </c>
-      <c r="D3" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B4" t="s">
         <v>108</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
+        <v>102</v>
+      </c>
+      <c r="D4" t="s">
         <v>109</v>
-      </c>
-      <c r="C4" t="s">
-        <v>103</v>
-      </c>
-      <c r="D4" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1657,10 +1672,10 @@
         <v>75</v>
       </c>
       <c r="C5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1671,52 +1686,52 @@
         <v>77</v>
       </c>
       <c r="C6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>112</v>
+      </c>
+      <c r="B7" t="s">
         <v>113</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D7" t="s">
         <v>114</v>
-      </c>
-      <c r="C7" t="s">
-        <v>103</v>
-      </c>
-      <c r="D7" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>115</v>
+      </c>
+      <c r="B8" t="s">
         <v>116</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
+        <v>102</v>
+      </c>
+      <c r="D8" t="s">
         <v>117</v>
-      </c>
-      <c r="C8" t="s">
-        <v>103</v>
-      </c>
-      <c r="D8" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>118</v>
+      </c>
+      <c r="B9" t="s">
         <v>119</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
+        <v>102</v>
+      </c>
+      <c r="D9" t="s">
         <v>120</v>
-      </c>
-      <c r="C9" t="s">
-        <v>103</v>
-      </c>
-      <c r="D9" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1727,24 +1742,24 @@
         <v>33</v>
       </c>
       <c r="C10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>122</v>
+      </c>
+      <c r="B11" t="s">
         <v>123</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
+        <v>102</v>
+      </c>
+      <c r="D11" t="s">
         <v>124</v>
-      </c>
-      <c r="C11" t="s">
-        <v>103</v>
-      </c>
-      <c r="D11" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -1752,41 +1767,41 @@
         <v>44</v>
       </c>
       <c r="B12" t="s">
+        <v>125</v>
+      </c>
+      <c r="C12" t="s">
+        <v>102</v>
+      </c>
+      <c r="D12" t="s">
         <v>126</v>
-      </c>
-      <c r="C12" t="s">
-        <v>103</v>
-      </c>
-      <c r="D12" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>127</v>
+      </c>
+      <c r="B13" t="s">
         <v>128</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
+        <v>102</v>
+      </c>
+      <c r="D13" t="s">
         <v>129</v>
-      </c>
-      <c r="C13" t="s">
-        <v>103</v>
-      </c>
-      <c r="D13" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>130</v>
+      </c>
+      <c r="B14" t="s">
         <v>131</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
+        <v>102</v>
+      </c>
+      <c r="D14" t="s">
         <v>132</v>
-      </c>
-      <c r="C14" t="s">
-        <v>103</v>
-      </c>
-      <c r="D14" t="s">
-        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -1913,10 +1928,10 @@
         <v>33</v>
       </c>
       <c r="C2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D2" t="s">
         <v>134</v>
-      </c>
-      <c r="D2" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -1927,10 +1942,10 @@
         <v>68</v>
       </c>
       <c r="C3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -1941,38 +1956,38 @@
         <v>75</v>
       </c>
       <c r="C4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>137</v>
+      </c>
+      <c r="B5" t="s">
         <v>138</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
+        <v>133</v>
+      </c>
+      <c r="D5" t="s">
         <v>139</v>
-      </c>
-      <c r="C5" t="s">
-        <v>134</v>
-      </c>
-      <c r="D5" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B6" t="s">
         <v>58</v>
       </c>
       <c r="C6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>
@@ -2007,72 +2022,72 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C2" t="s">
+        <v>151</v>
+      </c>
+      <c r="D2" t="s">
         <v>152</v>
-      </c>
-      <c r="D2" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C5" t="s">
         <v>151</v>
       </c>
-      <c r="C5" t="s">
-        <v>152</v>
-      </c>
       <c r="D5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C6" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -2107,58 +2122,58 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C2" t="s">
+        <v>187</v>
+      </c>
+      <c r="D2" t="s">
         <v>188</v>
-      </c>
-      <c r="D2" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D5" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -2166,153 +2181,153 @@
         <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B7" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C7" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B8" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C8" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B9" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C9" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B10" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C10" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D10" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C11" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D11" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B12" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C12" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D12" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B13" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C13" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B14" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B15" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C15" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D15" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B16" t="s">
+        <v>186</v>
+      </c>
+      <c r="C16" t="s">
         <v>187</v>
       </c>
-      <c r="C16" t="s">
-        <v>188</v>
-      </c>
       <c r="D16" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -2347,44 +2362,44 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B2" t="s">
         <v>75</v>
       </c>
       <c r="C2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>205</v>
+      </c>
+      <c r="B3" t="s">
         <v>206</v>
       </c>
-      <c r="B3" t="s">
-        <v>207</v>
-      </c>
       <c r="C3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B4" t="s">
         <v>77</v>
       </c>
       <c r="C4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -2395,52 +2410,52 @@
         <v>33</v>
       </c>
       <c r="C5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>212</v>
+      </c>
+      <c r="B6" t="s">
+        <v>214</v>
+      </c>
+      <c r="C6" t="s">
+        <v>204</v>
+      </c>
+      <c r="D6" t="s">
         <v>213</v>
-      </c>
-      <c r="B6" t="s">
-        <v>215</v>
-      </c>
-      <c r="C6" t="s">
-        <v>205</v>
-      </c>
-      <c r="D6" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>215</v>
+      </c>
+      <c r="B7" t="s">
         <v>216</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
+        <v>204</v>
+      </c>
+      <c r="D7" t="s">
         <v>217</v>
-      </c>
-      <c r="C7" t="s">
-        <v>205</v>
-      </c>
-      <c r="D7" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>218</v>
+      </c>
+      <c r="B8" t="s">
         <v>219</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
+        <v>204</v>
+      </c>
+      <c r="D8" t="s">
         <v>220</v>
-      </c>
-      <c r="C8" t="s">
-        <v>205</v>
-      </c>
-      <c r="D8" t="s">
-        <v>221</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added hagerstown, updated format of header in highest and best use doc
</commit_message>
<xml_diff>
--- a/Municipal_Zoning_Workbook.xlsx
+++ b/Municipal_Zoning_Workbook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/055abc5dbe1424b0/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="169" documentId="8_{3E8B709B-7093-42E6-92D8-1867EF89E086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE3BA393-8A6B-44F3-BDDA-BBC57A4AB012}"/>
+  <xr:revisionPtr revIDLastSave="214" documentId="8_{3E8B709B-7093-42E6-92D8-1867EF89E086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0635C5C-A150-4914-85D8-5FD7AD421CBB}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{CA185F06-9CD4-4691-B86E-FBA6669FCB7C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="8" xr2:uid="{CA185F06-9CD4-4691-B86E-FBA6669FCB7C}"/>
   </bookViews>
   <sheets>
     <sheet name="City of Frederick" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="Town of Poolesville" sheetId="6" r:id="rId6"/>
     <sheet name="City of Cumberland" sheetId="7" r:id="rId7"/>
     <sheet name="Town of Myersville" sheetId="8" r:id="rId8"/>
+    <sheet name="Hagerstown" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="240">
   <si>
     <t>Zone</t>
   </si>
@@ -724,6 +725,45 @@
   </si>
   <si>
     <t>Mixed-use Village (MXV-2)</t>
+  </si>
+  <si>
+    <t>Agricultural Transition</t>
+  </si>
+  <si>
+    <t>AT</t>
+  </si>
+  <si>
+    <t>City of Hagerstown Planning and Zoning Department</t>
+  </si>
+  <si>
+    <t>The purpose of the AT District is to enable agricultural uses to continue on newly annexed land, if desired by the property owner, as a temporary use until such time that the land is re-zoned for development. All lands within this district proposed for development shall be rezoned to another district to accommodate that development, in accordance with the policies and procedures set forth in this Article. The Planning Commission and the Mayor and City Council shall consider the policies and recommendations of the Comprehensive Plan when re-assigning zoning classification for AT land for development. When the property is to be given another classification, whether there was a mistake in assigning the AT classification and/or whether changes in the character of the neighborhood have occurred may be taken into consideration. However, a finding of mistake or change in character of the neighborhood shall not be required.</t>
+  </si>
+  <si>
+    <t>City Center - Mixed Use</t>
+  </si>
+  <si>
+    <t>CC-MU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The purpose of the CC-MU district is to promote development of a compact, pedestrian-oriented city center consisting of a diverse mix of residential, business, commercial, office, institutional, educational, and cultural and entertainment activities for workers, visitors, and residents; encourage pedestrian-oriented development within walking distance of transit opportunities at densities and intensities that will help to support transit usage and city center businesses; promote the health and well-being of residents by encouraging physical activity, alternative transportation, and greater social interaction; create a place that represents a unique, attractive, and memorable destination for visitors and residents; and enhance the community’s character through the promotion of high- quality urban design. </t>
+  </si>
+  <si>
+    <t>Commercial - Local</t>
+  </si>
+  <si>
+    <t>CL</t>
+  </si>
+  <si>
+    <t>The purpose of the CL district is to provide for the daily shopping and business needs of nearby residents and workers by permitting retail and service uses which are compatible in use and scale with the adjacent residential neighborhood.</t>
+  </si>
+  <si>
+    <t>CG</t>
+  </si>
+  <si>
+    <t>Commercial - General</t>
+  </si>
+  <si>
+    <t>The purpose of the CG district is to provide locations for businesses of a general nature to serve the community.</t>
   </si>
 </sst>
 </file>
@@ -2462,4 +2502,90 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3219F162-7BDF-486D-A2E2-BDD3A57DC069}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="47.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="255.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C2" t="s">
+        <v>229</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>231</v>
+      </c>
+      <c r="B3" t="s">
+        <v>232</v>
+      </c>
+      <c r="C3" t="s">
+        <v>229</v>
+      </c>
+      <c r="D3" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>234</v>
+      </c>
+      <c r="B4" t="s">
+        <v>235</v>
+      </c>
+      <c r="C4" t="s">
+        <v>229</v>
+      </c>
+      <c r="D4" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>238</v>
+      </c>
+      <c r="B5" t="s">
+        <v>237</v>
+      </c>
+      <c r="C5" t="s">
+        <v>229</v>
+      </c>
+      <c r="D5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>